<commit_message>
feat: create SOUM-DECO-3-Template.xlsx — clean sheet with all fixes
Created xlsx template with 4 tabs:
1. Products: all 62 current products (17 columns)
2. Orders: header only (15 columns incl. Variant column)
3. Stock: all 63 current stock entries with conditional formatting
   (red=0, yellow=1-3, green=>3)
4. Statistics: 5 sections with IFERROR-wrapped QUERY formulas
   - Summary (Total Orders, Revenue, Average Cart)
   - Top 10 Products (by count + revenue)
   - Top 10 Wilayas (by count + revenue)
   - Order Status Breakdown
   - Top 5 Wilayas by Revenue

All QUERY formulas wrapped in IFERROR to prevent #N/A errors
when Orders tab is empty.

Colored headers (brass #9A7E3A with white text), section headers
(sand #F1ECE3), title (cream #FAF8F4).
</commit_message>
<xml_diff>
--- a/download/SOUM-DECO-3-Template.xlsx
+++ b/download/SOUM-DECO-3-Template.xlsx
@@ -31,7 +31,7 @@
     <font>
       <name val="Inter"/>
       <b val="1"/>
-      <color rgb="001C1815"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -42,13 +42,13 @@
     <font>
       <name val="Inter"/>
       <b val="1"/>
-      <color rgb="001C1815"/>
+      <color rgb="009A7E3A"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Inter"/>
       <b val="1"/>
-      <color rgb="009A7E3A"/>
+      <color rgb="001C1815"/>
       <sz val="12"/>
     </font>
     <font>
@@ -66,8 +66,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8E4DC"/>
-        <bgColor rgb="00E8E4DC"/>
+        <fgColor rgb="009A7E3A"/>
+        <bgColor rgb="009A7E3A"/>
       </patternFill>
     </fill>
     <fill>
@@ -5243,8 +5243,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="350" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
-    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
     <col width="150" customWidth="1" min="4" max="4"/>
     <col width="150" customWidth="1" min="5" max="5"/>
   </cols>
@@ -5274,7 +5274,7 @@
         </is>
       </c>
       <c r="B4" s="8">
-        <f>COUNTA(Orders!C2:C)</f>
+        <f>IFERROR(COUNTA(Orders!C2:C),0)</f>
         <v/>
       </c>
     </row>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>SUM(Orders!G2:G)</f>
+        <f>IFERROR(SUM(Orders!G2:G),0)</f>
         <v/>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>IF(COUNTA(Orders!C2:C)&gt;0, SUM(Orders!G2:G)/COUNTA(Orders!C2:C), 0)</f>
+        <f>IFERROR(IF(COUNTA(Orders!C2:C)&gt;0,SUM(Orders!G2:G)/COUNTA(Orders!C2:C),0),0)</f>
         <v/>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
     </row>
     <row r="10">
       <c r="A10" s="10">
-        <f>QUERY(Orders!C2:G, "SELECT C, COUNT(C), SUM(G) WHERE C IS NOT NULL GROUP BY C ORDER BY COUNT(C) DESC LIMIT 10", 1)</f>
+        <f>IFERROR(QUERY(Orders!C2:G, "SELECT C, COUNT(C), SUM(G) WHERE C IS NOT NULL GROUP BY C ORDER BY COUNT(C) DESC LIMIT 10", 1), "Aucune commande")</f>
         <v/>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
     </row>
     <row r="24">
       <c r="A24" s="10">
-        <f>QUERY(Orders!J2:G, "SELECT J, COUNT(J), SUM(G) WHERE J IS NOT NULL GROUP BY J ORDER BY COUNT(J) DESC LIMIT 10", 1)</f>
+        <f>IFERROR(QUERY(Orders!J2:G, "SELECT J, COUNT(J), SUM(G) WHERE J IS NOT NULL GROUP BY J ORDER BY COUNT(J) DESC LIMIT 10", 1), "Aucune commande")</f>
         <v/>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
     </row>
     <row r="38">
       <c r="A38" s="10">
-        <f>QUERY(Orders!B2:B, "SELECT B, COUNT(B) WHERE B IS NOT NULL GROUP BY B ORDER BY COUNT(B) DESC LIMIT 10", 1)</f>
+        <f>IFERROR(QUERY(Orders!B2:B, "SELECT B, COUNT(B) WHERE B IS NOT NULL GROUP BY B ORDER BY COUNT(B) DESC LIMIT 10", 1), "Aucune commande")</f>
         <v/>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
     </row>
     <row r="52">
       <c r="A52" s="10">
-        <f>QUERY(Orders!J2:G, "SELECT J, SUM(G) WHERE J IS NOT NULL GROUP BY J ORDER BY SUM(G) DESC LIMIT 5", 1)</f>
+        <f>IFERROR(QUERY(Orders!J2:G, "SELECT J, SUM(G) WHERE J IS NOT NULL GROUP BY J ORDER BY SUM(G) DESC LIMIT 5", 1), "Aucune commande")</f>
         <v/>
       </c>
     </row>

</xml_diff>